<commit_message>
Simple Flow: SV-8183 FINAL report — add plain 'What needs to be done' beside every DEVIATION
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/sv8183/SimpleFlow_SV-8183_Permission-Test-FINAL-Report_2026-07-24.xlsx
+++ b/build/simple-flow/sv8183/SimpleFlow_SV-8183_Permission-Test-FINAL-Report_2026-07-24.xlsx
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -854,8 +854,9 @@
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -908,10 +909,15 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Related case (C-id + link)</t>
         </is>
@@ -958,10 +964,15 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
           <t>fe-route-probe.jsonl; be-settings-probe.json; residuals SM/SrSA/Foreman</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-01 = C29405 · https://shopview.testrail.io/index.php?/cases/view/29405 ; SF-PERM-06 = C29410 · https://shopview.testrail.io/index.php?/cases/view/29410</t>
         </is>
@@ -1008,10 +1019,15 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
           <t>element-matrix.json; residuals *_recvWO.png</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-02 = C29406 · https://shopview.testrail.io/index.php?/cases/view/29406 ; SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1058,10 +1074,15 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
           <t>residuals SM/SrSA/Foreman line controls</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1108,10 +1129,15 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
           <t>residuals FINDINGS (Complete disabled=data-state)</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1158,10 +1184,15 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
           <t>element-reobserve</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1208,10 +1239,15 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
           <t>Foreman_25777_*; TimeClock_25777_wizard.json; resolve-cores-endtoend.json</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-12 = C30647 · https://shopview.testrail.io/index.php?/cases/view/30647 (context); SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1258,10 +1294,15 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
           <t>tech-newpartrequest-dialog-2026-07-23.png</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-09 = C29413 · https://shopview.testrail.io/index.php?/cases/view/29413</t>
         </is>
@@ -1308,10 +1349,15 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
           <t>resolve-cores-endtoend.json</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1358,10 +1404,15 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
           <t>fe-route-probe.jsonl; residuals order controls</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-05 = C29409 · https://shopview.testrail.io/index.php?/cases/view/29409</t>
         </is>
@@ -1408,10 +1459,15 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
           <t>be-matrix-11roles.json; be-probe-batch1.json</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-05 = C29409 · https://shopview.testrail.io/index.php?/cases/view/29409 ; SF-PERM-03 = C29407 · https://shopview.testrail.io/index.php?/cases/view/29407</t>
         </is>
@@ -1458,10 +1514,15 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
+          <t>A view-only user can wrongly OPEN the Bulk Receive screen by ticking several orders and clicking 'Receive Selected' — they should not see that screen at all. The system still blocks the actual receiving, so no data is changed. The developer is already fixing this (ticket SV-8515, marked 'Ready to Fix'). QA action: no fix needed from us now — once the developer marks it fixed, re-test it: log in as a view-only user (Office role), open Bulk Receive, tick a few orders, click 'Receive Selected', and confirm that screen no longer opens for them.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
           <t>sv8515-bulk-receive-screen.png; sv8515-recv5-net.json (403)</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-11 = C30646 · https://shopview.testrail.io/index.php?/cases/view/30646 ; SF-PERM-03 = C29407 · https://shopview.testrail.io/index.php?/cases/view/29407</t>
         </is>
@@ -1508,10 +1569,15 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
           <t>be-matrix-11roles.json; order_Office.png (edit_note hidden)</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-03 = C29407 · https://shopview.testrail.io/index.php?/cases/view/29407</t>
         </is>
@@ -1558,10 +1624,15 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
           <t>rerun2 FINDINGS §2 (parts-catalogue routes per role)</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1608,10 +1679,15 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
           <t>rerun2 matrix (SFD-gated change-item)</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-03 = C29407 · https://shopview.testrail.io/index.php?/cases/view/29407</t>
         </is>
@@ -1658,10 +1734,15 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
           <t>markrev-*.png; residuals SM/SrSA/Foreman review</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-04 = C29408 · https://shopview.testrail.io/index.php?/cases/view/29408 ; SF-PERM-07 = C29411 · https://shopview.testrail.io/index.php?/cases/view/29411 ; SF-PERM-08 = C29412 · https://shopview.testrail.io/index.php?/cases/view/29412 ; SF-REV-09 = C29394 · https://shopview.testrail.io/index.php?/cases/view/29394</t>
         </is>
@@ -1708,10 +1789,15 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
           <t>§9.2 composition</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1758,10 +1844,15 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
           <t>§9.2 composition</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-10 = C29414 · https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
@@ -1808,10 +1899,15 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
           <t>sv8516-tc-menus.json; sv8516-tc-wo-lines.png</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-12 = C30647 · https://shopview.testrail.io/index.php?/cases/view/30647</t>
         </is>
@@ -2701,7 +2797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2709,7 +2805,8 @@
     <col width="52" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2747,6 +2844,11 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
           <t>Evidence</t>
         </is>
       </c>
@@ -2779,6 +2881,11 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
           <t>fe-route-probe.jsonl; be-settings-probe.json</t>
         </is>
       </c>
@@ -2811,6 +2918,11 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
           <t>element-matrix.json; residuals SM/SrSA/Foreman</t>
         </is>
       </c>
@@ -2843,6 +2955,11 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t>be-matrix-11roles.json; sv8515 reverify</t>
         </is>
       </c>
@@ -2875,6 +2992,11 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
           <t>markrev-*.png</t>
         </is>
       </c>
@@ -2907,6 +3029,11 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
           <t>fe-route-probe.jsonl; be-matrix (accept 403)</t>
         </is>
       </c>
@@ -2939,6 +3066,11 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
           <t>be-settings-probe.json; ticket dev comment</t>
         </is>
       </c>
@@ -2971,6 +3103,11 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
           <t>markrev-*.png (enabled SrSA/SA/PM; disabled SalesRep/Tech)</t>
         </is>
       </c>
@@ -3003,6 +3140,11 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
           <t>markrev-*.png + Milos ruling</t>
         </is>
       </c>
@@ -3035,6 +3177,11 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>tech-newpartrequest-dialog-2026-07-23.png</t>
         </is>
       </c>
@@ -3067,6 +3214,11 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
           <t>element-matrix.json (10/11 live); residuals</t>
         </is>
       </c>
@@ -3099,6 +3251,11 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
+          <t>A view-only user can wrongly OPEN the Bulk Receive screen by ticking several orders and clicking 'Receive Selected' — they should not see that screen at all. The system still blocks the actual receiving, so no data is changed. The developer is already fixing this (ticket SV-8515, marked 'Ready to Fix'). QA action: no fix needed from us now — once the developer marks it fixed, re-test it: log in as a view-only user (Office role), open Bulk Receive, tick a few orders, click 'Receive Selected', and confirm that screen no longer opens for them.</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
           <t>sv8515-bulk-receive-screen.png; sv8515-recv5-net.json (403)</t>
         </is>
       </c>
@@ -3131,6 +3288,11 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
           <t>sv8516-tc-menus.json; sv8516-tc-wo-lines.png</t>
         </is>
       </c>
@@ -3162,6 +3324,11 @@
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>markrev-*.png</t>
         </is>
@@ -3185,7 +3352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3193,9 +3360,10 @@
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3233,15 +3401,20 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
           <t>Spec cited (Rule 25)</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Covered by</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Was QA right?</t>
         </is>
@@ -3268,22 +3441,27 @@
           <t>On a clean Office role (25/25==template): per-PO button correctly hidden; BUT 'Receive Selected' DOES open the full editable /bulk-receive screen (33 inputs). Real receive fires accept -&gt; HTTP 403 'Access denied' — receive does NOT complete, no inventory mutated.</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>REAL FE-EXPOSURE DEVIATION — FE wrongly exposes an editable Bulk-Receive entry point to a view-only user; BE correctly blocks the receive. QA's 'receives same as Admin/bypass' is overstated (no escalation; write blocked 403). Inverse of Rule 24 = defect.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
+          <t>A view-only user can wrongly OPEN the Bulk Receive screen by ticking several orders and clicking 'Receive Selected' — they should not see that screen at all. The system still blocks the actual receiving, so no data is changed. The developer is already fixing this (ticket SV-8515, marked 'Ready to Fix'). QA action: no fix needed from us now — once the developer marks it fixed, re-test it: log in as a view-only user (Office role), open Bulk Receive, tick a few orders, click 'Receive Selected', and confirm that screen no longer opens for them.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
           <t>§9.1 'Bulk Receive page -&gt; Vendor &amp; Order Mgmt: Create &amp; Edit (route gate hasPartsPermissions)'; §9.2 Office Bulk Receive='No (4)', fn4 'View only -&gt; can open Bulk Receive but cannot receive'. BE matches spec; FE deviates.</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-11 = C30646 (VIU-Deviation)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>YES — real gap our first pass missed</t>
         </is>
@@ -3310,22 +3488,27 @@
           <t>Current build: Time Clock part kebab shows ONLY Return — Edit/Cancel/Change Vendor hidden (over-grant FE-fixed). BE part/change-request &amp; parts/delete=400 all roles (atom-collapse) -&gt; same edit possible via direct API.</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>FRONT-END FIXED. Residual 'same action via API' = PASS per Standing Rule 24 (FE blocks + BE/API allows = PASS; accepted ShopView model).</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
+          <t>No action needed — the developer has already fixed the front-end (the extra part-menu options are now hidden for this role). The only leftover is that the same change can still be made through the back-end interface, which company policy accepts. If you want, re-test after the next release to confirm the part menu still shows only 'Return'.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
           <t>§9.2 Time Clock='No' every column; Sasha: 'Users require WOL -&gt; Create &amp; Edit to manage part requests (make/edit/cancel)'. FE now enforces; BE atom-collapse (§9.4) spec-anticipated.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>SF-PERM-12 = C30647 (VIU-Verified, 'doable via API' flag in metadata)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>YES — real over-grant (now fixed)</t>
         </is>
@@ -3352,22 +3535,27 @@
           <t>Resolve-cores wizard FE-gated to completion-capable roles (Foreman operates it; Time Clock has no Complete button -&gt; unreachable). BE pre-resolve-cores=400 all roles (business-state, not 403) — not BE-permission-enforced. Return: inventory/returns/create=403 for SalesRep/Tech/TimeClock, reached-400 for Yes roles+Office; Returns page Parts-route-gated for negatives.</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>PRE-EXISTING, SPEC-ANTICIPATED (§9.4 atom-collapse SV-7864), NOT a Simple-Flow regression — same on Production. Under Rule 24 the FE-gated-but-BE-permissive resolve-core is a PASS. HELD pending Sasha's product ruling; not re-filed, not a new bug.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
+          <t>No fix needed from QA now — this behaves the same on the live Production site, so it is not a new Simple Flow break. It is waiting for the product team (Sasha) to decide the intended rule; once they do, re-test whether a user without the parts-editing permission can return a received special part and resolve cores, as ruled.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t>§9.1 'Resolve cores -&gt; WO Lines: Create &amp; Edit'; §9.4 'woOrderParts/workOrderLinesCreateAndEdit/woFullViewMode/woTechViewMode/workOrdersCreateAndEdit all resolve to ROLE_WORK_ORDER::VIEW+CREATE_AND_EDIT ... FE distinctions are conveniences, not BE-enforceable (SV-7864)'.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Held (SF-REV-14/C29399 &amp; SF-PERM-09/C29413 adjacent); no new case authored pending ruling</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>YES — real, correctly flagged as clarification</t>
         </is>

</xml_diff>